<commit_message>
sys_maturity: phase 2 operational manual layers 100 percent complete
</commit_message>
<xml_diff>
--- a/workflows/SMART_DEBT_TRACKER.xlsx
+++ b/workflows/SMART_DEBT_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arthu\GeminiEcosystem\workflows\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608087ED-144F-46A2-B157-3903FC442211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31041ADC-F86B-4475-98E0-9BEAD4E0F6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{F5A322B4-1A50-4262-8AA7-CD3191C5948E}"/>
   </bookViews>
@@ -505,6 +505,9 @@
       <c r="A3" s="1">
         <v>46163</v>
       </c>
+      <c r="B3">
+        <v>75</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1">

</xml_diff>